<commit_message>
jcb log edited to correct rate amount
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/JCB log/jcb log pahiro.xlsx
+++ b/बजेट माग estimate/JCB log/jcb log pahiro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\बजेट माग estimate\JCB log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D98C33-D610-463C-B16A-406836E9098F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45626ACA-78F8-47E3-B850-2D2F100D97F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ESTIMATE (3)" sheetId="1" state="hidden" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="7" sheetId="11" r:id="rId10"/>
     <sheet name="8" sheetId="12" r:id="rId11"/>
     <sheet name="9" sheetId="13" r:id="rId12"/>
-    <sheet name="month 4 and 5" sheetId="14" state="hidden" r:id="rId13"/>
+    <sheet name="month 4 and 5" sheetId="14" r:id="rId13"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId14"/>
@@ -67,7 +67,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">all!$A$1:$H$45</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'ESTIMATE (3)'!$A$1:$H$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'month 3'!$A$1:$H$34</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="12">'month 4 and 5'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="12">'month 4 and 5'!$A$1:$H$26</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'1'!$1:$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'2'!$1:$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'3'!$1:$9</definedName>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="71">
   <si>
     <t>सुरु घण्टा मिटर (क)</t>
   </si>
@@ -494,7 +494,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -597,6 +597,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1806,11 +1809,11 @@
         <v>2</v>
       </c>
       <c r="F10" s="30">
-        <v>3104</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>6208</v>
+        <v>4274</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>57</v>
@@ -1835,11 +1838,11 @@
         <v>4</v>
       </c>
       <c r="F11" s="30">
-        <v>3105</v>
+        <v>2137</v>
       </c>
       <c r="G11" s="1">
         <f>F11*E11</f>
-        <v>12420</v>
+        <v>8548</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>69</v>
@@ -1856,8 +1859,8 @@
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="2">
-        <f>SUM(G10:G10)</f>
-        <v>6208</v>
+        <f>SUM(G10:G11)</f>
+        <v>12822</v>
       </c>
       <c r="H12" s="3"/>
     </row>
@@ -1884,7 +1887,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>G12</f>
-        <v>6208</v>
+        <v>12822</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -1899,7 +1902,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>0.13*G14</f>
-        <v>807.04000000000008</v>
+        <v>1666.8600000000001</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -1914,7 +1917,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="2">
         <f>SUM(G14:G15)</f>
-        <v>7015.04</v>
+        <v>14488.86</v>
       </c>
       <c r="H16" s="3"/>
     </row>
@@ -2165,11 +2168,11 @@
         <v>7.2999999999999972</v>
       </c>
       <c r="F10" s="30">
-        <v>3103</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>22651.899999999991</v>
+        <v>15600.099999999993</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>70</v>
@@ -2187,7 +2190,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>22651.899999999991</v>
+        <v>15600.099999999993</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -2214,7 +2217,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>22651.899999999991</v>
+        <v>15600.099999999993</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -2229,7 +2232,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>2944.7469999999989</v>
+        <v>2028.0129999999992</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -2244,7 +2247,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>25596.64699999999</v>
+        <v>17628.112999999994</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -2495,11 +2498,11 @@
         <v>2</v>
       </c>
       <c r="F10" s="30">
-        <v>3102</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f>F10*E10</f>
-        <v>6204</v>
+        <v>4274</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>55</v>
@@ -2519,7 +2522,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>6204</v>
+        <v>4274</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -2546,7 +2549,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>6204</v>
+        <v>4274</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -2561,7 +2564,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>806.52</v>
+        <v>555.62</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -2576,7 +2579,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>7010.52</v>
+        <v>4829.62</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -2675,7 +2678,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A36A7736-3846-4BA4-9720-EF30AB2CCE9A}">
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="7" style="4" customWidth="1"/>
@@ -2827,11 +2830,11 @@
         <v>2</v>
       </c>
       <c r="F10" s="30">
-        <v>3102</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f>F10*E10</f>
-        <v>6204</v>
+        <v>4274</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>55</v>
@@ -2858,11 +2861,11 @@
         <v>7.2999999999999972</v>
       </c>
       <c r="F11" s="30">
-        <v>3103</v>
+        <v>2137</v>
       </c>
       <c r="G11" s="1">
         <f t="shared" ref="G11:G19" si="1">F11*E11</f>
-        <v>22651.899999999991</v>
+        <v>15600.099999999993</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>56</v>
@@ -2887,11 +2890,11 @@
         <v>2</v>
       </c>
       <c r="F12" s="30">
-        <v>3104</v>
+        <v>2137</v>
       </c>
       <c r="G12" s="1">
         <f t="shared" si="1"/>
-        <v>6208</v>
+        <v>4274</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>57</v>
@@ -2916,11 +2919,11 @@
         <v>4</v>
       </c>
       <c r="F13" s="30">
-        <v>3105</v>
+        <v>2137</v>
       </c>
       <c r="G13" s="1">
         <f t="shared" si="1"/>
-        <v>12420</v>
+        <v>8548</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>58</v>
@@ -2945,11 +2948,11 @@
         <v>6</v>
       </c>
       <c r="F14" s="30">
-        <v>3110</v>
+        <v>2137</v>
       </c>
       <c r="G14" s="1">
         <f t="shared" si="1"/>
-        <v>18660</v>
+        <v>12822</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>60</v>
@@ -2974,11 +2977,11 @@
         <v>5</v>
       </c>
       <c r="F15" s="30">
-        <v>3111</v>
+        <v>2137</v>
       </c>
       <c r="G15" s="1">
         <f t="shared" si="1"/>
-        <v>15555</v>
+        <v>10685</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>61</v>
@@ -3003,11 +3006,11 @@
         <v>7</v>
       </c>
       <c r="F16" s="30">
-        <v>3112</v>
+        <v>2137</v>
       </c>
       <c r="G16" s="1">
         <f t="shared" si="1"/>
-        <v>21784</v>
+        <v>14959</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>61</v>
@@ -3032,11 +3035,11 @@
         <v>6</v>
       </c>
       <c r="F17" s="30">
-        <v>3113</v>
+        <v>2137</v>
       </c>
       <c r="G17" s="1">
         <f t="shared" si="1"/>
-        <v>18678</v>
+        <v>12822</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>62</v>
@@ -3061,11 +3064,11 @@
         <v>7</v>
       </c>
       <c r="F18" s="30">
-        <v>3102</v>
+        <v>2137</v>
       </c>
       <c r="G18" s="1">
         <f t="shared" si="1"/>
-        <v>21714</v>
+        <v>14959</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>63</v>
@@ -3090,11 +3093,11 @@
         <v>8</v>
       </c>
       <c r="F19" s="30">
-        <v>3102</v>
+        <v>2137</v>
       </c>
       <c r="G19" s="1">
         <f t="shared" si="1"/>
-        <v>24816</v>
+        <v>17096</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>63</v>
@@ -3112,9 +3115,9 @@
       <c r="F20" s="8"/>
       <c r="G20" s="2">
         <f>SUM(G10:G19)</f>
-        <v>168690.9</v>
-      </c>
-      <c r="H20" s="3"/>
+        <v>116039.09999999999</v>
+      </c>
+      <c r="H20" s="41"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="1"/>
@@ -3139,7 +3142,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="2">
         <f>G20</f>
-        <v>168690.9</v>
+        <v>116039.09999999999</v>
       </c>
       <c r="H22" s="3"/>
     </row>
@@ -3154,7 +3157,7 @@
       <c r="F23" s="8"/>
       <c r="G23" s="2">
         <f>0.13*G22</f>
-        <v>21929.816999999999</v>
+        <v>15085.082999999999</v>
       </c>
       <c r="H23" s="3"/>
     </row>
@@ -3169,7 +3172,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="2">
         <f>SUM(G22:G23)</f>
-        <v>190620.717</v>
+        <v>131124.18299999999</v>
       </c>
       <c r="H24" s="3"/>
     </row>
@@ -3182,74 +3185,26 @@
       <c r="G25" s="14"/>
       <c r="H25" s="12"/>
     </row>
-    <row r="28" spans="1:10" ht="20.25">
-      <c r="B28" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="E28" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="H28" s="24" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="20.25">
-      <c r="B29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="H29" s="25"/>
-    </row>
-    <row r="30" spans="1:10" ht="18.75">
-      <c r="B30" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="E30" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="H30" s="26" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="35" spans="3:6" ht="20.25">
-      <c r="C35" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="F35" s="24" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" spans="3:6" ht="20.25">
-      <c r="C36" s="25"/>
-      <c r="F36" s="25"/>
-    </row>
-    <row r="37" spans="3:6" ht="18.75">
-      <c r="C37" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="D37" s="27"/>
-      <c r="F37" s="26" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="42" spans="3:6">
-      <c r="C42" s="4" t="s">
+    <row r="31" spans="1:10">
+      <c r="C31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D31" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="E31" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="3:6">
-      <c r="C43" s="4" t="s">
+    <row r="32" spans="1:10">
+      <c r="C32" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D32" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E43" s="4" t="str">
-        <f>E42</f>
+      <c r="E32" s="4" t="str">
+        <f>E31</f>
         <v>without vat</v>
       </c>
     </row>
@@ -3261,8 +3216,11 @@
     <mergeCell ref="A5:H5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="1" right="0.25" top="1" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="70" fitToHeight="2" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -4567,11 +4525,11 @@
         <v>8</v>
       </c>
       <c r="F10" s="30">
-        <v>3102</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>24816</v>
+        <v>17096</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>63</v>
@@ -4589,7 +4547,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>24816</v>
+        <v>17096</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -4616,7 +4574,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>24816</v>
+        <v>17096</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -4631,7 +4589,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>3226.08</v>
+        <v>2222.48</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -4646,7 +4604,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>28042.080000000002</v>
+        <v>19318.48</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -4897,11 +4855,11 @@
         <v>7</v>
       </c>
       <c r="F10" s="30">
-        <v>3102</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>21714</v>
+        <v>14959</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>63</v>
@@ -4919,7 +4877,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>21714</v>
+        <v>14959</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -4946,7 +4904,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>21714</v>
+        <v>14959</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -4961,7 +4919,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>2822.82</v>
+        <v>1944.67</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -4976,7 +4934,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>24536.82</v>
+        <v>16903.669999999998</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -5227,11 +5185,11 @@
         <v>6</v>
       </c>
       <c r="F10" s="30">
-        <v>3113</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>18678</v>
+        <v>12822</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>66</v>
@@ -5249,7 +5207,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>18678</v>
+        <v>12822</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -5276,7 +5234,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>18678</v>
+        <v>12822</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -5291,7 +5249,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>2428.14</v>
+        <v>1666.8600000000001</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -5306,7 +5264,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>21106.14</v>
+        <v>14488.86</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -5557,11 +5515,11 @@
         <v>7</v>
       </c>
       <c r="F10" s="30">
-        <v>3112</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>21784</v>
+        <v>14959</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>67</v>
@@ -5579,7 +5537,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>21784</v>
+        <v>14959</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -5606,7 +5564,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>21784</v>
+        <v>14959</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -5621,7 +5579,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>2831.92</v>
+        <v>1944.67</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -5636,7 +5594,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>24615.919999999998</v>
+        <v>16903.669999999998</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -5887,11 +5845,11 @@
         <v>5</v>
       </c>
       <c r="F10" s="30">
-        <v>3111</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" ref="G10" si="1">F10*E10</f>
-        <v>15555</v>
+        <v>10685</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>68</v>
@@ -5909,7 +5867,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>15555</v>
+        <v>10685</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -5936,7 +5894,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>15555</v>
+        <v>10685</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -5951,7 +5909,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>2022.15</v>
+        <v>1389.05</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -5966,7 +5924,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>17577.150000000001</v>
+        <v>12074.05</v>
       </c>
       <c r="H15" s="3"/>
     </row>
@@ -6217,11 +6175,11 @@
         <v>6</v>
       </c>
       <c r="F10" s="30">
-        <v>3110</v>
+        <v>2137</v>
       </c>
       <c r="G10" s="1">
         <f>F10*E10</f>
-        <v>18660</v>
+        <v>12822</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>60</v>
@@ -6239,7 +6197,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="2">
         <f>SUM(G10:G10)</f>
-        <v>18660</v>
+        <v>12822</v>
       </c>
       <c r="H11" s="3"/>
     </row>
@@ -6266,7 +6224,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="2">
         <f>G11</f>
-        <v>18660</v>
+        <v>12822</v>
       </c>
       <c r="H13" s="3"/>
     </row>
@@ -6281,7 +6239,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="2">
         <f>0.13*G13</f>
-        <v>2425.8000000000002</v>
+        <v>1666.8600000000001</v>
       </c>
       <c r="H14" s="3"/>
     </row>
@@ -6296,7 +6254,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="2">
         <f>SUM(G13:G14)</f>
-        <v>21085.8</v>
+        <v>14488.86</v>
       </c>
       <c r="H15" s="3"/>
     </row>

</xml_diff>